<commit_message>
docs: literature review sheet — add the named prior-FYP finding
Merges Shahoud's 2026-09-06 archive check (risk-register R39) into
Sheet 1 and Sheet 5: S24-011-D-HDLM, Hallucination Detection in Language
Model Textual Responses (Spring 2024), the closest match found across
all 660 titles in the 12 published department cohorts.

Same underlying problem (untrustworthy AI output, no error signal) but
scoped to one LLM's text output, not a multi-agent execution trace —
roughly one of Granite's four pipeline stages. Keeps the sheet consistent
with the same merge already made in the v2 deck and the design canvas.
</commit_message>
<xml_diff>
--- a/markdowns/03-market-and-literature-research/Literature_Review_Sheet.xlsx
+++ b/markdowns/03-market-and-literature-research/Literature_Review_Sheet.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="247">
   <si>
     <t>Granite — Literature Review, in one place</t>
   </si>
@@ -57,6 +57,12 @@
     <t>Across all seven papers, none tests transfer to a multi-agent architecture that was never used in its own benchmark construction. That gap survived full-text reading of every paper.</t>
   </si>
   <si>
+    <t>Closest prior FYP in the department</t>
+  </si>
+  <si>
+    <t>S24-011-D-HDLM, 'Hallucination Detection in Language Model Textual Responses' (Spring 2024). Same underlying problem — untrustworthy AI output with no error signal — but scoped to one LLM's text, not a multi-agent execution trace. Covers roughly one of our four pipeline stages. Detail on Sheet 5.</t>
+  </si>
+  <si>
     <t>How to use this workbook</t>
   </si>
   <si>
@@ -673,6 +679,15 @@
   </si>
   <si>
     <t>15-20% deliberately clean controls in our own benchmark, with a provisional target under 5%. This is what stops 'flag everything' from looking like success.</t>
+  </si>
+  <si>
+    <t>6. No prior departmental FYP covers this</t>
+  </si>
+  <si>
+    <t>Checked against all 660 titles across the 12 published cohorts, Spring-2019 to Fall-2025, structurally rather than by title. Closest match found: S24-011-D-HDLM, 'Hallucination Detection in Language Model Textual Responses' (Spring 2024) — identified in Shahoud's archive check, risk-register R39.</t>
+  </si>
+  <si>
+    <t>That project confirms the underlying problem is real and department-recognised, but it detects hallucinations in ONE LLM's text output. No agent or step attribution, no propagation-path modelling, no repair or replay step — roughly one of Granite's four pipeline stages. Name it before a panel asks you to.</t>
   </si>
   <si>
     <t>5. Step-level attribution is far from solved</t>
@@ -834,17 +849,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFE3EFF1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFF7EFDC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1E242F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE3EFF1"/>
       </patternFill>
     </fill>
     <fill>
@@ -880,7 +895,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -907,13 +922,19 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -922,10 +943,10 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1292,7 +1313,7 @@
   <sheetPr>
     <tabColor rgb="FFC89B3C"/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1358,19 +1379,19 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+    <row r="10" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="3"/>
-    </row>
-    <row r="12" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+      <c r="B10" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="5" t="s">
+    </row>
+    <row r="12" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
         <v>15</v>
       </c>
+      <c r="B12" s="3"/>
     </row>
     <row r="13" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
@@ -1404,26 +1425,34 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
+    <row r="17" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="3"/>
-    </row>
-    <row r="19" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
+      <c r="B17" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="9" t="s">
+    </row>
+    <row r="19" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
         <v>26</v>
       </c>
+      <c r="B19" s="3"/>
     </row>
     <row r="20" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="11" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="21" ht="46" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1431,8 +1460,8 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A19:B19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1458,7 +1487,7 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1470,7 +1499,7 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1482,211 +1511,211 @@
     </row>
     <row r="3" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" s="10" t="s">
+      <c r="A4" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="B4" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="C4" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="D4" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="E4" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="F4" s="12" t="s">
         <v>38</v>
       </c>
+      <c r="G4" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="5" ht="112" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C5" s="12" t="s">
+      <c r="A5" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="B5" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="C5" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="D5" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="G5" s="12" t="s">
+      <c r="E5" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="H5" s="12" t="s">
+      <c r="F5" s="14" t="s">
         <v>46</v>
       </c>
+      <c r="G5" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="H5" s="14" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="6" ht="112" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="C6" s="12" t="s">
+      <c r="A6" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="B6" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="C6" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="D6" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="G6" s="12" t="s">
+      <c r="E6" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="H6" s="12" t="s">
+      <c r="F6" s="14" t="s">
         <v>54</v>
       </c>
+      <c r="G6" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="H6" s="14" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="7" ht="112" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="C7" s="14" t="s">
+      <c r="A7" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="B7" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="C7" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="D7" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="E7" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="F7" s="16" t="s">
         <v>62</v>
       </c>
+      <c r="G7" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="8" ht="112" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="C8" s="14" t="s">
+      <c r="A8" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="B8" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="C8" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="D8" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="G8" s="14" t="s">
+      <c r="E8" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="H8" s="14" t="s">
+      <c r="F8" s="16" t="s">
         <v>70</v>
       </c>
+      <c r="G8" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="H8" s="16" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="9" ht="112" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="B9" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="D9" s="16" t="s">
+      <c r="A9" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="B9" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="F9" s="16" t="s">
+      <c r="C9" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="D9" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="G9" s="16" t="s">
+      <c r="E9" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="H9" s="16" t="s">
+      <c r="F9" s="18" t="s">
         <v>77</v>
       </c>
+      <c r="G9" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="H9" s="18" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="10" ht="112" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
-        <v>78</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="E10" s="14" t="s">
+      <c r="A10" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="B10" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="D10" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="G10" s="14" t="s">
+      <c r="E10" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="H10" s="14" t="s">
+      <c r="F10" s="16" t="s">
         <v>83</v>
       </c>
+      <c r="G10" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="H10" s="16" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="11" ht="112" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="D11" s="14" t="s">
+      <c r="A11" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="B11" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="C11" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="D11" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="G11" s="14" t="s">
+      <c r="E11" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="H11" s="14" t="s">
+      <c r="F11" s="16" t="s">
         <v>90</v>
+      </c>
+      <c r="G11" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="H11" s="16" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -1718,7 +1747,7 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1728,7 +1757,7 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1738,128 +1767,128 @@
     </row>
     <row r="3" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="E4" s="10" t="s">
+      <c r="A4" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="B4" s="12" t="s">
         <v>96</v>
       </c>
+      <c r="C4" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="5" ht="42" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="C5" s="18" t="s">
+      <c r="A5" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="B5" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="C5" s="20" t="s">
         <v>101</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="D5" s="20" t="s">
         <v>102</v>
       </c>
+      <c r="E5" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="F5" s="20" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>99</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="E6" s="13" t="s">
+      <c r="A6" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="B6" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="D6" s="16" t="s">
         <v>106</v>
       </c>
+      <c r="E6" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>99</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>99</v>
-      </c>
-      <c r="E7" s="13" t="s">
+      <c r="A7" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="B7" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7" s="16" t="s">
         <v>110</v>
       </c>
+      <c r="D7" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="B8" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>99</v>
-      </c>
-      <c r="D8" s="16" t="s">
+      <c r="A8" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="E8" s="15" t="s">
+      <c r="B8" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="F8" s="16" t="s">
+      <c r="C8" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="D8" s="18" t="s">
         <v>115</v>
       </c>
+      <c r="E8" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="F8" s="18" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="19" t="s">
-        <v>116</v>
-      </c>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
+      <c r="A10" s="21" t="s">
+        <v>118</v>
+      </c>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
     </row>
     <row r="11" ht="66" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
+      <c r="A11" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
     </row>
     <row r="13" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -1868,83 +1897,83 @@
       <c r="F13" s="3"/>
     </row>
     <row r="14" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="C14" s="10" t="s">
+      <c r="A14" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="B14" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="C14" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="F14" s="10" t="s">
+      <c r="D14" s="12" t="s">
         <v>124</v>
       </c>
+      <c r="E14" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="15" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="C15" s="14" t="s">
+      <c r="A15" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="D15" s="14" t="s">
-        <v>114</v>
-      </c>
-      <c r="E15" s="14" t="s">
+      <c r="B15" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="F15" s="14" t="s">
+      <c r="C15" s="16" t="s">
         <v>129</v>
       </c>
+      <c r="D15" s="16" t="s">
+        <v>116</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>130</v>
+      </c>
+      <c r="F15" s="16" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="16" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="E16" s="16" t="s">
         <v>130</v>
       </c>
-      <c r="B16" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="F16" s="14" t="s">
-        <v>133</v>
+      <c r="F16" s="16" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="17" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="17" t="s">
-        <v>134</v>
-      </c>
-      <c r="B17" s="18" t="s">
-        <v>135</v>
-      </c>
-      <c r="C17" s="18" t="s">
+      <c r="A17" s="19" t="s">
         <v>136</v>
       </c>
-      <c r="D17" s="18" t="s">
-        <v>101</v>
-      </c>
-      <c r="E17" s="18" t="s">
+      <c r="B17" s="20" t="s">
         <v>137</v>
       </c>
-      <c r="F17" s="18" t="s">
+      <c r="C17" s="20" t="s">
         <v>138</v>
+      </c>
+      <c r="D17" s="20" t="s">
+        <v>103</v>
+      </c>
+      <c r="E17" s="20" t="s">
+        <v>139</v>
+      </c>
+      <c r="F17" s="20" t="s">
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -1978,7 +2007,7 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1989,7 +2018,7 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2000,233 +2029,233 @@
     </row>
     <row r="3" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="C4" s="10" t="s">
+      <c r="A4" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="B4" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="E4" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="F4" s="10" t="s">
+      <c r="C4" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="D4" s="12" t="s">
         <v>146</v>
       </c>
+      <c r="E4" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="5" ht="78" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>147</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>148</v>
-      </c>
-      <c r="D5" s="18" t="s">
+      <c r="A5" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>149</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="C5" s="20" t="s">
         <v>150</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="D5" s="20" t="s">
         <v>151</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="19" t="s">
         <v>152</v>
       </c>
+      <c r="F5" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="G5" s="20" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="6" ht="78" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
-        <v>153</v>
-      </c>
-      <c r="B6" s="18" t="s">
-        <v>154</v>
-      </c>
-      <c r="C6" s="18" t="s">
+      <c r="A6" s="19" t="s">
         <v>155</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="B6" s="20" t="s">
         <v>156</v>
       </c>
-      <c r="E6" s="17" t="s">
-        <v>150</v>
-      </c>
-      <c r="F6" s="18" t="s">
+      <c r="C6" s="20" t="s">
         <v>157</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="D6" s="20" t="s">
         <v>158</v>
       </c>
+      <c r="E6" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="F6" s="20" t="s">
+        <v>159</v>
+      </c>
+      <c r="G6" s="20" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="7" ht="78" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="17" t="s">
-        <v>159</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>154</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>160</v>
-      </c>
-      <c r="D7" s="18" t="s">
+      <c r="A7" s="19" t="s">
         <v>161</v>
       </c>
-      <c r="E7" s="17" t="s">
-        <v>150</v>
-      </c>
-      <c r="F7" s="18" t="s">
+      <c r="B7" s="20" t="s">
+        <v>156</v>
+      </c>
+      <c r="C7" s="20" t="s">
         <v>162</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="D7" s="20" t="s">
         <v>163</v>
       </c>
+      <c r="E7" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="F7" s="20" t="s">
+        <v>164</v>
+      </c>
+      <c r="G7" s="20" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="8" ht="78" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
-        <v>164</v>
-      </c>
-      <c r="B8" s="22" t="s">
-        <v>165</v>
-      </c>
-      <c r="C8" s="22" t="s">
+      <c r="A8" s="23" t="s">
         <v>166</v>
       </c>
-      <c r="D8" s="22" t="s">
+      <c r="B8" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="E8" s="21" t="s">
+      <c r="C8" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="F8" s="22" t="s">
+      <c r="D8" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="G8" s="22" t="s">
+      <c r="E8" s="23" t="s">
         <v>170</v>
       </c>
+      <c r="F8" s="24" t="s">
+        <v>171</v>
+      </c>
+      <c r="G8" s="24" t="s">
+        <v>172</v>
+      </c>
     </row>
     <row r="9" ht="78" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>172</v>
-      </c>
-      <c r="C9" s="14" t="s">
+      <c r="A9" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="B9" s="16" t="s">
         <v>174</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="C9" s="16" t="s">
         <v>175</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="D9" s="16" t="s">
         <v>176</v>
       </c>
-      <c r="G9" s="14" t="s">
+      <c r="E9" s="15" t="s">
         <v>177</v>
       </c>
+      <c r="F9" s="16" t="s">
+        <v>178</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="10" ht="78" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>154</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="D10" s="14" t="s">
+      <c r="A10" s="15" t="s">
         <v>180</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="B10" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="C10" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="D10" s="16" t="s">
         <v>182</v>
       </c>
-      <c r="G10" s="14" t="s">
+      <c r="E10" s="15" t="s">
         <v>183</v>
       </c>
+      <c r="F10" s="16" t="s">
+        <v>184</v>
+      </c>
+      <c r="G10" s="16" t="s">
+        <v>185</v>
+      </c>
     </row>
     <row r="11" ht="78" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="13" t="s">
-        <v>184</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>154</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="D11" s="14" t="s">
+      <c r="A11" s="15" t="s">
         <v>186</v>
       </c>
-      <c r="E11" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="F11" s="14" t="s">
+      <c r="B11" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="C11" s="16" t="s">
         <v>187</v>
       </c>
-      <c r="G11" s="14" t="s">
+      <c r="D11" s="16" t="s">
         <v>188</v>
       </c>
+      <c r="E11" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="F11" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="G11" s="16" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="12" ht="78" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="15" t="s">
-        <v>189</v>
-      </c>
-      <c r="B12" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>190</v>
-      </c>
-      <c r="D12" s="16" t="s">
+      <c r="A12" s="17" t="s">
         <v>191</v>
       </c>
-      <c r="E12" s="15" t="s">
+      <c r="B12" s="18" t="s">
+        <v>156</v>
+      </c>
+      <c r="C12" s="18" t="s">
         <v>192</v>
       </c>
-      <c r="F12" s="16" t="s">
+      <c r="D12" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="G12" s="16" t="s">
+      <c r="E12" s="17" t="s">
         <v>194</v>
       </c>
+      <c r="F12" s="18" t="s">
+        <v>195</v>
+      </c>
+      <c r="G12" s="18" t="s">
+        <v>196</v>
+      </c>
     </row>
     <row r="13" ht="78" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
-        <v>195</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>196</v>
-      </c>
-      <c r="C13" s="12" t="s">
+      <c r="A13" s="13" t="s">
         <v>197</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="B13" s="14" t="s">
         <v>198</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="C13" s="14" t="s">
         <v>199</v>
       </c>
-      <c r="F13" s="12" t="s">
+      <c r="D13" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="G13" s="12" t="s">
+      <c r="E13" s="13" t="s">
         <v>201</v>
+      </c>
+      <c r="F13" s="14" t="s">
+        <v>202</v>
+      </c>
+      <c r="G13" s="14" t="s">
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -2245,7 +2274,7 @@
   <sheetPr>
     <tabColor rgb="FFA8760F"/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -2254,97 +2283,108 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
     </row>
     <row r="3" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>205</v>
-      </c>
-      <c r="C4" s="10" t="s">
+      <c r="A4" s="12" t="s">
         <v>206</v>
       </c>
+      <c r="B4" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>208</v>
+      </c>
     </row>
     <row r="5" ht="108" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
-        <v>207</v>
-      </c>
-      <c r="B5" s="16" t="s">
-        <v>208</v>
-      </c>
-      <c r="C5" s="16" t="s">
+      <c r="A5" s="17" t="s">
         <v>209</v>
       </c>
+      <c r="B5" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>211</v>
+      </c>
     </row>
     <row r="6" ht="108" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
-        <v>210</v>
-      </c>
-      <c r="B6" s="16" t="s">
-        <v>211</v>
-      </c>
-      <c r="C6" s="16" t="s">
+      <c r="A6" s="17" t="s">
         <v>212</v>
       </c>
+      <c r="B6" s="18" t="s">
+        <v>213</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>214</v>
+      </c>
     </row>
     <row r="7" ht="108" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
-        <v>213</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>214</v>
-      </c>
-      <c r="C7" s="14" t="s">
+      <c r="A7" s="15" t="s">
         <v>215</v>
       </c>
+      <c r="B7" s="16" t="s">
+        <v>216</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="8" ht="108" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
-        <v>216</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>217</v>
-      </c>
-      <c r="C8" s="14" t="s">
+      <c r="A8" s="15" t="s">
         <v>218</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>219</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="9" ht="108" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="11" ht="52" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="23" t="s">
-        <v>222</v>
-      </c>
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
+        <v>223</v>
+      </c>
+    </row>
+    <row r="10" ht="108" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="15" t="s">
+        <v>224</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>225</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="12" ht="52" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="25" t="s">
+        <v>227</v>
+      </c>
+      <c r="B12" s="25"/>
+      <c r="C12" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A12:C12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2367,7 +2407,7 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2375,7 +2415,7 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2383,124 +2423,124 @@
     </row>
     <row r="3" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>225</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>226</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>227</v>
+      <c r="A4" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="5" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>228</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>229</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>230</v>
+      <c r="A5" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>233</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>234</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="6" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>228</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>231</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>232</v>
+      <c r="A6" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>233</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>236</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="7" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>228</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="14" t="s">
+      <c r="A7" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="B7" s="16" t="s">
         <v>233</v>
       </c>
+      <c r="C7" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>238</v>
+      </c>
     </row>
     <row r="8" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>228</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="D8" s="14" t="s">
-        <v>234</v>
+      <c r="A8" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>233</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="9" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="B9" s="16" t="s">
-        <v>228</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>235</v>
-      </c>
-      <c r="D9" s="16" t="s">
-        <v>236</v>
+      <c r="A9" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>240</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="10" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
-        <v>78</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>237</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>238</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>239</v>
+      <c r="A10" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>242</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>243</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="11" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>237</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>238</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>240</v>
+      <c r="A11" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>242</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>243</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="24" t="s">
-        <v>241</v>
-      </c>
-      <c r="B13" s="24"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
+      <c r="A13" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>